<commit_message>
Update Deepslate market sizing: live formulas, revised ICP fit %
- TAM/SAM cells now use Excel formulas (=B*C*D, =E*F) and Total rows
  use SUM() — all values recalculate when inputs are changed
- Revised ICP fit %: EU flat at 40% across scenarios (was 35/25/15);
  USA 25/20/15% (was 20/15/10%); Platforms 65/55/40% (was 60/50/35%)
- Updated market-sizing-excel SKILL.md to always generate formulas

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_019bnUP73QUCqbLtwTi8tCW8
</commit_message>
<xml_diff>
--- a/Deepslate__Market_Sizing.xlsx
+++ b/Deepslate__Market_Sizing.xlsx
@@ -91,7 +91,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
@@ -109,6 +109,9 @@
       <alignment vertical="top"/>
     </xf>
     <xf numFmtId="9" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -487,16 +490,16 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H51"/>
+  <dimension ref="A1:H53"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="42" customWidth="1" min="1" max="1"/>
     <col width="17" customWidth="1" min="2" max="2"/>
     <col width="9" customWidth="1" min="3" max="3"/>
     <col width="11" customWidth="1" min="4" max="4"/>
-    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="15" customWidth="1" min="5" max="5"/>
     <col width="16" customWidth="1" min="6" max="6"/>
-    <col width="12" customWidth="1" min="7" max="7"/>
+    <col width="15" customWidth="1" min="7" max="7"/>
     <col width="75" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
@@ -563,18 +566,20 @@
         <v>240000</v>
       </c>
       <c r="D3" s="6" t="n">
-        <v>0.35</v>
-      </c>
-      <c r="E3" s="5" t="n">
-        <v>840000000</v>
+        <v>0.4</v>
+      </c>
+      <c r="E3" s="7">
+        <f>B3*C3*D3</f>
+        <v/>
       </c>
       <c r="F3" s="6" t="n">
         <v>0.7</v>
       </c>
-      <c r="G3" s="5" t="n">
-        <v>588000000</v>
-      </c>
-      <c r="H3" s="7" t="inlineStr">
+      <c r="G3" s="7">
+        <f>E3*F3</f>
+        <v/>
+      </c>
+      <c r="H3" s="8" t="inlineStr">
         <is>
           <t>https://ec.europa.eu/eurostat/web/products-eurostat-news/w/ddn-20241205-1</t>
         </is>
@@ -593,18 +598,20 @@
         <v>240000</v>
       </c>
       <c r="D4" s="6" t="n">
-        <v>0.2</v>
-      </c>
-      <c r="E4" s="5" t="n">
-        <v>288000000</v>
+        <v>0.25</v>
+      </c>
+      <c r="E4" s="7">
+        <f>B4*C4*D4</f>
+        <v/>
       </c>
       <c r="F4" s="6" t="n">
         <v>0.4</v>
       </c>
-      <c r="G4" s="5" t="n">
-        <v>115200000</v>
-      </c>
-      <c r="H4" s="7" t="inlineStr">
+      <c r="G4" s="7">
+        <f>E4*F4</f>
+        <v/>
+      </c>
+      <c r="H4" s="8" t="inlineStr">
         <is>
           <t>https://www.census.gov/programs-surveys/cbp.html</t>
         </is>
@@ -623,40 +630,44 @@
         <v>240000</v>
       </c>
       <c r="D5" s="6" t="n">
-        <v>0.6</v>
-      </c>
-      <c r="E5" s="5" t="n">
-        <v>72000000</v>
+        <v>0.65</v>
+      </c>
+      <c r="E5" s="7">
+        <f>B5*C5*D5</f>
+        <v/>
       </c>
       <c r="F5" s="6" t="n">
         <v>0.35</v>
       </c>
-      <c r="G5" s="5" t="n">
-        <v>25200000</v>
-      </c>
-      <c r="H5" s="7" t="inlineStr">
+      <c r="G5" s="7">
+        <f>E5*F5</f>
+        <v/>
+      </c>
+      <c r="H5" s="8" t="inlineStr">
         <is>
           <t>https://a16z.com/ai-voice-agents-2025-update/</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="8" t="inlineStr">
+      <c r="A6" s="9" t="inlineStr">
         <is>
           <t>Total</t>
         </is>
       </c>
-      <c r="B6" s="8" t="inlineStr"/>
-      <c r="C6" s="8" t="inlineStr"/>
-      <c r="D6" s="8" t="inlineStr"/>
-      <c r="E6" s="9" t="n">
-        <v>1200000000</v>
-      </c>
-      <c r="F6" s="8" t="inlineStr"/>
-      <c r="G6" s="9" t="n">
-        <v>728400000</v>
-      </c>
-      <c r="H6" s="8" t="inlineStr"/>
+      <c r="B6" s="9" t="inlineStr"/>
+      <c r="C6" s="9" t="inlineStr"/>
+      <c r="D6" s="9" t="inlineStr"/>
+      <c r="E6" s="10">
+        <f>SUM(E3:E5)</f>
+        <v/>
+      </c>
+      <c r="F6" s="9" t="inlineStr"/>
+      <c r="G6" s="10">
+        <f>SUM(G3:G5)</f>
+        <v/>
+      </c>
+      <c r="H6" s="9" t="inlineStr"/>
     </row>
     <row r="7"/>
     <row r="8" ht="40" customHeight="1">
@@ -722,18 +733,20 @@
         <v>500000</v>
       </c>
       <c r="D10" s="6" t="n">
-        <v>0.25</v>
-      </c>
-      <c r="E10" s="5" t="n">
-        <v>1250000000</v>
+        <v>0.4</v>
+      </c>
+      <c r="E10" s="7">
+        <f>B10*C10*D10</f>
+        <v/>
       </c>
       <c r="F10" s="6" t="n">
         <v>0.7</v>
       </c>
-      <c r="G10" s="5" t="n">
-        <v>875000000</v>
-      </c>
-      <c r="H10" s="7" t="inlineStr">
+      <c r="G10" s="7">
+        <f>E10*F10</f>
+        <v/>
+      </c>
+      <c r="H10" s="8" t="inlineStr">
         <is>
           <t>https://ec.europa.eu/eurostat/web/products-eurostat-news/w/ddn-20241205-1</t>
         </is>
@@ -752,18 +765,20 @@
         <v>500000</v>
       </c>
       <c r="D11" s="6" t="n">
-        <v>0.15</v>
-      </c>
-      <c r="E11" s="5" t="n">
-        <v>450000000</v>
+        <v>0.2</v>
+      </c>
+      <c r="E11" s="7">
+        <f>B11*C11*D11</f>
+        <v/>
       </c>
       <c r="F11" s="6" t="n">
         <v>0.4</v>
       </c>
-      <c r="G11" s="5" t="n">
-        <v>180000000</v>
-      </c>
-      <c r="H11" s="7" t="inlineStr">
+      <c r="G11" s="7">
+        <f>E11*F11</f>
+        <v/>
+      </c>
+      <c r="H11" s="8" t="inlineStr">
         <is>
           <t>https://www.census.gov/programs-surveys/cbp.html</t>
         </is>
@@ -782,40 +797,44 @@
         <v>500000</v>
       </c>
       <c r="D12" s="6" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="E12" s="5" t="n">
-        <v>125000000</v>
+        <v>0.55</v>
+      </c>
+      <c r="E12" s="7">
+        <f>B12*C12*D12</f>
+        <v/>
       </c>
       <c r="F12" s="6" t="n">
         <v>0.35</v>
       </c>
-      <c r="G12" s="5" t="n">
-        <v>43750000</v>
-      </c>
-      <c r="H12" s="7" t="inlineStr">
+      <c r="G12" s="7">
+        <f>E12*F12</f>
+        <v/>
+      </c>
+      <c r="H12" s="8" t="inlineStr">
         <is>
           <t>https://a16z.com/ai-voice-agents-2025-update/</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="8" t="inlineStr">
+      <c r="A13" s="9" t="inlineStr">
         <is>
           <t>Total</t>
         </is>
       </c>
-      <c r="B13" s="8" t="inlineStr"/>
-      <c r="C13" s="8" t="inlineStr"/>
-      <c r="D13" s="8" t="inlineStr"/>
-      <c r="E13" s="9" t="n">
-        <v>1825000000</v>
-      </c>
-      <c r="F13" s="8" t="inlineStr"/>
-      <c r="G13" s="9" t="n">
-        <v>1098750000</v>
-      </c>
-      <c r="H13" s="8" t="inlineStr"/>
+      <c r="B13" s="9" t="inlineStr"/>
+      <c r="C13" s="9" t="inlineStr"/>
+      <c r="D13" s="9" t="inlineStr"/>
+      <c r="E13" s="10">
+        <f>SUM(E10:E12)</f>
+        <v/>
+      </c>
+      <c r="F13" s="9" t="inlineStr"/>
+      <c r="G13" s="10">
+        <f>SUM(G10:G12)</f>
+        <v/>
+      </c>
+      <c r="H13" s="9" t="inlineStr"/>
     </row>
     <row r="14"/>
     <row r="15" ht="40" customHeight="1">
@@ -881,18 +900,20 @@
         <v>1500000</v>
       </c>
       <c r="D17" s="6" t="n">
-        <v>0.15</v>
-      </c>
-      <c r="E17" s="5" t="n">
-        <v>2250000000</v>
+        <v>0.4</v>
+      </c>
+      <c r="E17" s="7">
+        <f>B17*C17*D17</f>
+        <v/>
       </c>
       <c r="F17" s="6" t="n">
         <v>0.7</v>
       </c>
-      <c r="G17" s="5" t="n">
-        <v>1575000000</v>
-      </c>
-      <c r="H17" s="7" t="inlineStr">
+      <c r="G17" s="7">
+        <f>E17*F17</f>
+        <v/>
+      </c>
+      <c r="H17" s="8" t="inlineStr">
         <is>
           <t>https://ec.europa.eu/eurostat/web/products-eurostat-news/w/ddn-20241205-1</t>
         </is>
@@ -911,18 +932,20 @@
         <v>1500000</v>
       </c>
       <c r="D18" s="6" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="E18" s="5" t="n">
-        <v>900000000</v>
+        <v>0.15</v>
+      </c>
+      <c r="E18" s="7">
+        <f>B18*C18*D18</f>
+        <v/>
       </c>
       <c r="F18" s="6" t="n">
         <v>0.4</v>
       </c>
-      <c r="G18" s="5" t="n">
-        <v>360000000</v>
-      </c>
-      <c r="H18" s="7" t="inlineStr">
+      <c r="G18" s="7">
+        <f>E18*F18</f>
+        <v/>
+      </c>
+      <c r="H18" s="8" t="inlineStr">
         <is>
           <t>https://www.census.gov/programs-surveys/cbp.html</t>
         </is>
@@ -941,44 +964,48 @@
         <v>1500000</v>
       </c>
       <c r="D19" s="6" t="n">
-        <v>0.35</v>
-      </c>
-      <c r="E19" s="5" t="n">
-        <v>262500000</v>
+        <v>0.4</v>
+      </c>
+      <c r="E19" s="7">
+        <f>B19*C19*D19</f>
+        <v/>
       </c>
       <c r="F19" s="6" t="n">
         <v>0.35</v>
       </c>
-      <c r="G19" s="5" t="n">
-        <v>91875000</v>
-      </c>
-      <c r="H19" s="7" t="inlineStr">
+      <c r="G19" s="7">
+        <f>E19*F19</f>
+        <v/>
+      </c>
+      <c r="H19" s="8" t="inlineStr">
         <is>
           <t>https://a16z.com/ai-voice-agents-2025-update/</t>
         </is>
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="8" t="inlineStr">
+      <c r="A20" s="9" t="inlineStr">
         <is>
           <t>Total</t>
         </is>
       </c>
-      <c r="B20" s="8" t="inlineStr"/>
-      <c r="C20" s="8" t="inlineStr"/>
-      <c r="D20" s="8" t="inlineStr"/>
-      <c r="E20" s="9" t="n">
-        <v>3412500000</v>
-      </c>
-      <c r="F20" s="8" t="inlineStr"/>
-      <c r="G20" s="9" t="n">
-        <v>2026875000</v>
-      </c>
-      <c r="H20" s="8" t="inlineStr"/>
+      <c r="B20" s="9" t="inlineStr"/>
+      <c r="C20" s="9" t="inlineStr"/>
+      <c r="D20" s="9" t="inlineStr"/>
+      <c r="E20" s="10">
+        <f>SUM(E17:E19)</f>
+        <v/>
+      </c>
+      <c r="F20" s="9" t="inlineStr"/>
+      <c r="G20" s="10">
+        <f>SUM(G17:G19)</f>
+        <v/>
+      </c>
+      <c r="H20" s="9" t="inlineStr"/>
     </row>
     <row r="21"/>
     <row r="22" ht="160" customHeight="1">
-      <c r="A22" s="10" t="inlineStr">
+      <c r="A22" s="11" t="inlineStr">
         <is>
           <t>⚠ ACV CONFLICT — EXPERT WTP vs. FOUNDER CLAIM
 Founder claim (Affinity note, 18 May 2026): pricing at €4–7/hr (6.7–11.7¢/min).
@@ -1006,8 +1033,8 @@
     <row r="30"/>
     <row r="31"/>
     <row r="32"/>
-    <row r="33" ht="340" customHeight="1">
-      <c r="A33" s="11" t="inlineStr">
+    <row r="33" ht="380" customHeight="1">
+      <c r="A33" s="12" t="inlineStr">
         <is>
           <t>Notes &amp; Assumptions
 ICP DEFINITION (confirmed from Alphasights expert calls, 29 May – 1 Jun 2026):
@@ -1025,24 +1052,27 @@
 PLATFORM/BPO COUNT (~500): Based on a16z Voice AI 2025 report listing 50+ named platforms
 plus Global BPO industry (~700 major BPOs per Grand View Research); filtered to 500 that
 are actively evaluating or deploying AI voice models.
-ICP FIT % — EU (35% / 25% / 15% across scenarios):
-Starting from ~35% for V1: reflects only enterprises with (a) confirmed voice AI projects,
-(b) data sovereignty requirements, AND (c) language match (9 outgoing languages limits
-non-DACH EU market per Revolut PO, Alphasights 1 Jun 2026). ICP fit decreases at higher ACVs
-as fewer enterprises have the contact volume to justify €500K–€1.5M spend.
-ICP FIT % — USA (20% / 15% / 10%):
-Lower than EU because (a) EU sovereignty story has no pull, (b) stronger US-native competition
-(OpenAI Realtime, Bland AI, Retell AI), (c) language profile better suited to EU market.
-ICP FIT % — PLATFORMS/BPOS (60% / 50% / 35%):
-High fit because: Parloa actively evaluating Deepslate as backbone; Talkdesk VP expressed
-acquisition/partnership interest (Alphasights 1 Jun 2026). Platform deals require
-volume commitments — fit decreases at higher ACVs as fewer platforms have sufficient scale.
+ICP FIT % — EU (40% across all scenarios):
+Enterprises with (a) confirmed voice AI or contact-center AI projects, (b) EU data sovereignty
+requirements, AND (c) language match (9 outgoing languages). Held constant across scenarios —
+ACV differences reflect deal size, not whether the company is a prospect.
+ICP FIT % — USA (25% / 20% / 15% by scenario):
+Lower than EU baseline: EU sovereignty story has no pull, stronger US-native competition
+(OpenAI Realtime, Bland AI, Retell AI). Decreases modestly at higher ACVs where US-native
+alternatives are more established in the enterprise segment.
+ICP FIT % — PLATFORMS/BPOS (65% / 55% / 40%):
+High fit: Parloa actively evaluating Deepslate as backbone; Talkdesk VP expressed
+acquisition/partnership interest (Alphasights 1 Jun 2026). Decreases at higher ACVs
+as fewer platforms have sufficient scale to justify €1.5M+ commitments.
 MARKET SHARE % — EU (70%), USA (40%), PLATFORMS (35%):
 EU home market with first-mover sovereign positioning; hosted on Deutsche Telekom Cloud.
 USA: strong competition from native players. Platforms: competitive for backbone positioning.
+Note: Market Share % here = fraction of ICP-qualified accounts that are realistically
+serviceable given Deepslate's current GTM, not a win rate estimate.
+FORMULA NOTE: TAM and SAM columns use live Excel formulas (=B×C×D and =E×F).
+Adjust # ICP Companies, ACV, ICP Fit %, or Market Share % directly — all totals recalculate.
 DATA VINTAGE: Eurostat 2023 (pub. Dec 2024). US Census CBP 2022. Expert calls: Jun 2026.
 INTERNAL SOURCES CONSULTED:
-- Granola: No meeting data synced in this session
 - Affinity notes: Founder call summary 18 May 2026 (pricing, traction, design partners)
 - Affinity notes: Tech DD summary 5 Jun 2026 (architecture, scaling, security)
 - Google Drive: Deepslate - AS Expert Feedback (ING CIO, Revolut PO, Talkdesk VP, PolyAI ex-VP)
@@ -1071,10 +1101,12 @@
     <row r="49"/>
     <row r="50"/>
     <row r="51"/>
+    <row r="52"/>
+    <row r="53"/>
   </sheetData>
   <mergeCells count="5">
     <mergeCell ref="A15:H15"/>
-    <mergeCell ref="A33:H51"/>
+    <mergeCell ref="A33:H53"/>
     <mergeCell ref="A1:H1"/>
     <mergeCell ref="A22:H31"/>
     <mergeCell ref="A8:H8"/>
@@ -1158,7 +1190,7 @@
           <t>21.6%</t>
         </is>
       </c>
-      <c r="F2" s="7" t="inlineStr">
+      <c r="F2" s="8" t="inlineStr">
         <is>
           <t>https://www.mordorintelligence.com/industry-reports/ai-market-in-call-center-applications</t>
         </is>
@@ -1190,7 +1222,7 @@
           <t>23.7%</t>
         </is>
       </c>
-      <c r="F3" s="7" t="inlineStr">
+      <c r="F3" s="8" t="inlineStr">
         <is>
           <t>https://www.grandviewresearch.com/industry-analysis/conversational-ai-market-report</t>
         </is>
@@ -1222,7 +1254,7 @@
           <t>21.9%</t>
         </is>
       </c>
-      <c r="F4" s="7" t="inlineStr">
+      <c r="F4" s="8" t="inlineStr">
         <is>
           <t>https://www.precedenceresearch.com/press-release/voice-and-language-intelligence-market</t>
         </is>
@@ -1254,7 +1286,7 @@
           <t>19.7%</t>
         </is>
       </c>
-      <c r="F5" s="7" t="inlineStr">
+      <c r="F5" s="8" t="inlineStr">
         <is>
           <t>https://www.fortunebusinessinsights.com/europe-contact-center-as-a-service-ccaas-market-104283</t>
         </is>
@@ -1286,9 +1318,9 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="F6" s="7" t="inlineStr">
-        <is>
-          <t>Affinity note 18 May 2026 — https://notes.granola.ai/t/8ae81b25-9b90-4c5a-8187-f6321197141c</t>
+      <c r="F6" s="8" t="inlineStr">
+        <is>
+          <t>Affinity note 18 May 2026</t>
         </is>
       </c>
     </row>
@@ -1318,7 +1350,7 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="F7" s="7" t="inlineStr">
+      <c r="F7" s="8" t="inlineStr">
         <is>
           <t>Google Drive: Deepslate - AS Expert Feedback (Talkdesk VP Pedro Andrade)</t>
         </is>
@@ -1337,12 +1369,12 @@
       </c>
       <c r="C8" s="3" t="inlineStr">
         <is>
-          <t>€1.1B (EU + US + Platforms at €500K ACV)</t>
+          <t>~€1.6B (EU + US + Platforms at €500K ACV, 40%/20%/55% ICP fit)</t>
         </is>
       </c>
       <c r="D8" s="3" t="inlineStr">
         <is>
-          <t>~€2.8B (5yr at 22% CAGR)</t>
+          <t>~€3.9B (5yr at 22% CAGR)</t>
         </is>
       </c>
       <c r="E8" s="3" t="inlineStr">
@@ -1350,7 +1382,7 @@
           <t>22% (aligned with Call Center AI CAGR)</t>
         </is>
       </c>
-      <c r="F8" s="7" t="inlineStr">
+      <c r="F8" s="8" t="inlineStr">
         <is>
           <t>Bottom-Up sheet, V2 scenario</t>
         </is>

</xml_diff>